<commit_message>
Examen A asterisco terminado
</commit_message>
<xml_diff>
--- a/Evalucacion A asterisco.xlsx
+++ b/Evalucacion A asterisco.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\richa\Documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1EA106D-12FE-4A0D-9D4D-94855A9633DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8561C17D-ED94-40F7-9654-FB24E7E83859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{138929AC-8231-4B42-8E0B-E9E77F8E4102}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Comienzo</t>
   </si>
@@ -132,7 +132,25 @@
     <t>G118 H50 F168 46</t>
   </si>
   <si>
-    <t>G114 H40 F154 47</t>
+    <t>G118 H30 F148 48</t>
+  </si>
+  <si>
+    <t>G128 H40 F164 47</t>
+  </si>
+  <si>
+    <t>G132 H30 F162 56</t>
+  </si>
+  <si>
+    <t>G132 H10 F142 58</t>
+  </si>
+  <si>
+    <t>G142 H20 F162 57</t>
+  </si>
+  <si>
+    <t>G146 H10 F156 50</t>
+  </si>
+  <si>
+    <t>G142 H0 F142 59</t>
   </si>
   <si>
     <r>
@@ -448,45 +466,315 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>,37,38,46,</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>47</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>,55,56</t>
-    </r>
-  </si>
-  <si>
-    <t>G128 H40 F168 55</t>
-  </si>
-  <si>
-    <t>G124 H30 F154 56</t>
-  </si>
-  <si>
-    <t>14,23,32,31,33,13,22,15,24,4,6,3,7,2,11,20,29,38,47,56</t>
+      <t>,37,</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>38</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,46,47,</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>48</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,56,57,</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>58</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,49,50,</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>59</t>
+    </r>
+  </si>
+  <si>
+    <t>G142 H20 F162 49</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,14,23,32,31,33,13,22,15,24,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,6,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,7,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>11</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>29</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>38</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>48</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>58</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>59</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -502,8 +790,15 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color theme="0"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -512,6 +807,13 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -555,7 +857,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -569,10 +871,19 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -904,22 +1215,22 @@
       <c r="B2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>15</v>
       </c>
       <c r="F2" s="3">
         <v>5</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="5" t="s">
         <v>17</v>
       </c>
       <c r="I2" s="2" t="s">
@@ -931,32 +1242,32 @@
       <c r="L2" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
+      <c r="M2" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
     </row>
     <row r="3" spans="2:18" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D3" s="4">
         <v>12</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="5" t="s">
         <v>10</v>
       </c>
       <c r="H3" s="4">
@@ -972,7 +1283,7 @@
         <v>3</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
@@ -984,19 +1295,19 @@
       <c r="B4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>25</v>
       </c>
       <c r="D4" s="4">
         <v>21</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="5" t="s">
         <v>13</v>
       </c>
       <c r="H4" s="4">
@@ -1013,19 +1324,19 @@
       <c r="B5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>27</v>
       </c>
       <c r="D5" s="4">
         <v>30</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="5" t="s">
         <v>9</v>
       </c>
       <c r="H5" s="4">
@@ -1042,7 +1353,7 @@
       <c r="B6" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>30</v>
       </c>
       <c r="D6" s="4">
@@ -1075,16 +1386,16 @@
         <v>31</v>
       </c>
       <c r="C7" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="2">
-        <v>48</v>
-      </c>
-      <c r="E7" s="2">
-        <v>49</v>
-      </c>
-      <c r="F7" s="2">
-        <v>50</v>
+      <c r="E7" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="G7" s="2">
         <v>51</v>
@@ -1103,20 +1414,20 @@
       </c>
     </row>
     <row r="8" spans="2:18" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="2">
+        <v>55</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="D8" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="2">
-        <v>57</v>
-      </c>
-      <c r="E8" s="2">
-        <v>58</v>
-      </c>
-      <c r="F8" s="5">
-        <v>59</v>
+      <c r="F8" s="9" t="s">
+        <v>38</v>
       </c>
       <c r="G8" s="2">
         <v>60</v>

</xml_diff>